<commit_message>
Adds vehicle vintaging in the transportation sector.
</commit_message>
<xml_diff>
--- a/InputData/plcy-schd/V/Vintage.xlsx
+++ b/InputData/plcy-schd/V/Vintage.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DanO'Brien\Models\EPS\US\eps-us\InputData\plcy-schd\V\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\plcy-schd\V\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD12AEC6-80C9-4241-9904-9376C77E7216}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B08ED24-DC89-437E-A97B-D921200BCD2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="29925" yWindow="1125" windowWidth="21600" windowHeight="11175" activeTab="5" xr2:uid="{70679913-52CE-4866-92D3-04053F7F27F8}"/>
+    <workbookView xWindow="1125" yWindow="1125" windowWidth="43200" windowHeight="17145" activeTab="6" xr2:uid="{70679913-52CE-4866-92D3-04053F7F27F8}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -19,6 +19,7 @@
     <sheet name="CV" sheetId="6" r:id="rId4"/>
     <sheet name="PV" sheetId="7" r:id="rId5"/>
     <sheet name="HV" sheetId="8" r:id="rId6"/>
+    <sheet name="VV" sheetId="9" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>Source: None</t>
   </si>
@@ -61,9 +62,6 @@
     <t>Vintage</t>
   </si>
   <si>
-    <t>FV First Vintage</t>
-  </si>
-  <si>
     <t>Current Vintage</t>
   </si>
   <si>
@@ -77,6 +75,18 @@
   </si>
   <si>
     <t>Vintage1950</t>
+  </si>
+  <si>
+    <t>First Vehicle Vintage (oldest model year tracked in the vehicle stock; earlier vehicles are lumped into it)</t>
+  </si>
+  <si>
+    <t>Last Vehicle Vintage: must equal FINAL TIME (plcy-schd/FT), or vehicles sold after it never enter the stock</t>
+  </si>
+  <si>
+    <t>FV First Vintage; HV Historical Vintage; CV, PV Current and Preceding Vintage; VV Vehicle Vintage (added 2026-09-28)</t>
+  </si>
+  <si>
+    <t>Vehicle Vintage</t>
   </si>
 </sst>
 </file>
@@ -464,7 +474,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6602441D-D56C-41AD-B87E-E90087615EB8}">
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -474,7 +484,7 @@
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>7</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -504,6 +514,22 @@
       </c>
       <c r="B10" s="1" t="s">
         <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A11">
+        <v>1965</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12">
+        <v>2050</v>
+      </c>
+      <c r="B12" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
@@ -1445,7 +1471,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -1469,7 +1495,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -2387,7 +2413,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
@@ -3305,12 +3331,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -3736,4 +3762,535 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A696C8A4-4301-4750-9FE9-BEFA4FB39A6B}">
+  <dimension ref="A1:A87"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1965</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1966</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1967</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1968</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1969</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1970</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1971</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1972</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1973</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1974</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A12" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1975</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A13" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1976</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1977</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1978</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1979</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1980</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1981</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1982</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A20" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1983</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A21" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1984</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1985</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1986</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1987</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1988</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1989</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1990</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1991</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1992</v>
+      </c>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A30" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1993</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A31" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1994</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1995</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1996</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1997</v>
+      </c>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage1999</v>
+      </c>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2002</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2003</v>
+      </c>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2004</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2005</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2006</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2007</v>
+      </c>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2008</v>
+      </c>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2009</v>
+      </c>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2010</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2011</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2012</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2013</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2014</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2015</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2016</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2017</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2018</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A56" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2019</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2020</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2021</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2022</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2023</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2024</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2025</v>
+      </c>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2026</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2027</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2028</v>
+      </c>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A66" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2029</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A67" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2030</v>
+      </c>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A68" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2031</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A69" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2032</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A70" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2033</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A71" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2034</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A72" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2035</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A73" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2036</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A74" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2037</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A75" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2038</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A76" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2039</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A77" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2040</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A78" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2041</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A79" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2042</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A80" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2043</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A81" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2044</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A82" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2045</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A83" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2046</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A84" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2047</v>
+      </c>
+    </row>
+    <row r="85" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A85" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2048</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A86" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2049</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A87" t="str">
+        <f>IF(ROW()-1&gt;About!$A$12-About!$A$11+1,"","Vintage"&amp;(About!$A$11+ROW()-2))</f>
+        <v>Vintage2050</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>